<commit_message>
Auto sync 2026-10-20 13:54:22
</commit_message>
<xml_diff>
--- a/outputs/logistics-review/OMS状态-导出验收.xlsx
+++ b/outputs/logistics-review/OMS状态-导出验收.xlsx
@@ -330,7 +330,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 13:53:36</t>
+          <t xml:space="preserve">2026-10-24 13:54:01</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -378,12 +378,12 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:53:36</t>
+          <t xml:space="preserve">2026-10-20 13:54:00</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:53:42</t>
+          <t xml:space="preserve">2026-10-20 13:54:06</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -396,7 +396,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-22 09:53:36</t>
+          <t xml:space="preserve">2026-10-22 09:54:01</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -406,12 +406,12 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 12:53:36</t>
+          <t xml:space="preserve">2026-10-20 12:54:01</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 12:53:36</t>
+          <t xml:space="preserve">2026-10-20 12:54:01</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19 13:53:36</t>
+          <t xml:space="preserve">2026-10-19 13:54:01</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -622,12 +622,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 13:53:36</t>
+          <t xml:space="preserve">2026-10-24 13:54:01</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:53:31</t>
+          <t xml:space="preserve">2026-10-20 13:53:56</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:53:37</t>
+          <t xml:space="preserve">2026-10-20 13:54:02</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19 13:53:36</t>
+          <t xml:space="preserve">2026-10-19 13:54:01</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -717,12 +717,12 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 13:53:36</t>
+          <t xml:space="preserve">2026-10-24 13:54:01</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:53:31</t>
+          <t xml:space="preserve">2026-10-20 13:53:56</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:53:37</t>
+          <t xml:space="preserve">2026-10-20 13:54:02</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19 13:53:36</t>
+          <t xml:space="preserve">2026-10-19 13:54:01</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 13:53:36</t>
+          <t xml:space="preserve">2026-10-24 13:54:01</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:53:36</t>
+          <t xml:space="preserve">2026-10-20 13:54:00</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:53:42</t>
+          <t xml:space="preserve">2026-10-20 13:54:06</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19 13:53:36</t>
+          <t xml:space="preserve">2026-10-19 13:54:01</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -907,12 +907,12 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 13:53:36</t>
+          <t xml:space="preserve">2026-10-24 13:54:01</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:53:36</t>
+          <t xml:space="preserve">2026-10-20 13:54:00</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:53:42</t>
+          <t xml:space="preserve">2026-10-20 13:54:06</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">

</xml_diff>